<commit_message>
Adresslisten überarbeitet: Richter Aluminium raus, Logistiker verkleinert
- Zielgruppe 1: Referenzkunde Richter Aluminium entfernt (36 Einträge)
- Zielgruppe 2: Großkonzerne und Netzwerkspediteure (DACHSER, Rhenus,
  Hellmann, Emons, Logwin, Fiege, LOXXESS, BLG, Arvato, Schnellecke,
  Gebrüder Weiss, Raben u.a.) ersetzt durch kleinere, inhabergeführte
  Speditionen und Kontraktlogistiker mit Mandantenlager (31 Einträge)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KugR1U5dxR4p4yhkLqU2yh
</commit_message>
<xml_diff>
--- a/adresslisten/Zielgruppe_1_Industrieunternehmen_SCM.xlsx
+++ b/adresslisten/Zielgruppe_1_Industrieunternehmen_SCM.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Industrieunternehmen" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Industrieunternehmen'!$A$1:$C$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Industrieunternehmen'!$A$1:$C$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -471,634 +471,617 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Richter Aluminium GmbH</t>
+          <t>OTTO FUCHS KG</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://www.richter-aluminium.com</t>
+          <t>https://www.otto-fuchs.com</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>+49 781 28416-0</t>
+          <t>+49 2354 73-0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>OTTO FUCHS KG</t>
+          <t>Erbslöh Aluminium GmbH</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://www.otto-fuchs.com</t>
+          <t>https://www.erbsloeh.de</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>+49 2354 73-0</t>
+          <t>+49 2053 95-0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Erbslöh Aluminium GmbH</t>
+          <t>Wieland-Werke AG</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://www.erbsloeh.de</t>
+          <t>https://www.wieland.com</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>+49 2053 95-0</t>
+          <t>+49 731 944-0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Wieland-Werke AG</t>
+          <t>Hammerer Aluminium Industries GmbH</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.wieland.com</t>
+          <t>https://www.hai-aluminium.com</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>+49 731 944-0</t>
+          <t>+43 7722 891-0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Hammerer Aluminium Industries GmbH</t>
+          <t>AMAG Austria Metall AG</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://www.hai-aluminium.com</t>
+          <t>https://www.amag.at</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>+43 7722 891-0</t>
+          <t>+43 7722 801-0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AMAG Austria Metall AG</t>
+          <t>Constellium Singen GmbH</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>https://www.amag.at</t>
+          <t>https://www.constellium.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>+43 7722 801-0</t>
+          <t>+49 7731 80-0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Constellium Singen GmbH</t>
+          <t>Gebrüder Meiser GmbH</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>https://www.constellium.com</t>
+          <t>https://www.meiser.de</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>+49 7731 80-0</t>
+          <t>+49 6887 309-0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Gebrüder Meiser GmbH</t>
+          <t>KIRCHHOFF Automotive Deutschland GmbH</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>https://www.meiser.de</t>
+          <t>https://www.kirchhoff-automotive.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>+49 6887 309-0</t>
+          <t>+49 2722 696-0</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>KIRCHHOFF Automotive Deutschland GmbH</t>
+          <t>PWO AG (Progress-Werk Oberkirch)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>https://www.kirchhoff-automotive.com</t>
+          <t>https://www.pwo-group.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>+49 2722 696-0</t>
+          <t>+49 7802 84-0</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PWO AG (Progress-Werk Oberkirch)</t>
+          <t>ElringKlinger AG</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>https://www.pwo-group.com</t>
+          <t>https://www.elringklinger.de</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>+49 7802 84-0</t>
+          <t>+49 7123 724-0</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ElringKlinger AG</t>
+          <t>Eberspächer Gruppe GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://www.elringklinger.de</t>
+          <t>https://www.eberspaecher.com</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>+49 7123 724-0</t>
+          <t>+49 711 939-00</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Eberspächer Gruppe GmbH &amp; Co. KG</t>
+          <t>SIMONA AG</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>https://www.eberspaecher.com</t>
+          <t>https://www.simona.de</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>+49 711 939-00</t>
+          <t>+49 6752 14-0</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>SIMONA AG</t>
+          <t>Pöppelmann GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>https://www.simona.de</t>
+          <t>https://www.poeppelmann.com</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>+49 6752 14-0</t>
+          <t>+49 4442 982-0</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Pöppelmann GmbH &amp; Co. KG</t>
+          <t>Röchling SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>https://www.poeppelmann.com</t>
+          <t>https://www.roechling.com</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>+49 4442 982-0</t>
+          <t>+49 621 4402-0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Röchling SE &amp; Co. KG</t>
+          <t>igus GmbH</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>https://www.roechling.com</t>
+          <t>https://www.igus.de</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>+49 621 4402-0</t>
+          <t>+49 2203 9649-0</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>igus GmbH</t>
+          <t>Weidmüller Interface GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>https://www.igus.de</t>
+          <t>https://www.weidmueller.de</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>+49 2203 9649-0</t>
+          <t>+49 5231 14-0</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Weidmüller Interface GmbH &amp; Co. KG</t>
+          <t>HARTING Stiftung &amp; Co. KG</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>https://www.weidmueller.de</t>
+          <t>https://www.harting.com</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>+49 5231 14-0</t>
+          <t>+49 5772 47-0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HARTING Stiftung &amp; Co. KG</t>
+          <t>WAGO GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>https://www.harting.com</t>
+          <t>https://www.wago.com</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>+49 5772 47-0</t>
+          <t>+49 571 887-0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>WAGO GmbH &amp; Co. KG</t>
+          <t>Lapp Holding SE</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>https://www.wago.com</t>
+          <t>https://www.lapp.com</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>+49 571 887-0</t>
+          <t>+49 711 7838-01</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Lapp Holding SE</t>
+          <t>Rösler Oberflächentechnik GmbH</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>https://www.lapp.com</t>
+          <t>https://www.rosler.com</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>+49 711 7838-01</t>
+          <t>+49 9533 924-0</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Rösler Oberflächentechnik GmbH</t>
+          <t>Schmitz Cargobull AG</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>https://www.rosler.com</t>
+          <t>https://www.cargobull.com</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>+49 9533 924-0</t>
+          <t>+49 2558 81-0</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Schmitz Cargobull AG</t>
+          <t>Kögel Trailer GmbH</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>https://www.cargobull.com</t>
+          <t>https://www.koegel.com</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>+49 2558 81-0</t>
+          <t>+49 8285 88-0</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Kögel Trailer GmbH</t>
+          <t>Bernard KRONE Holding SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>https://www.koegel.com</t>
+          <t>https://www.krone-group.com</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>+49 8285 88-0</t>
+          <t>+49 5977 935-0</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Bernard KRONE Holding SE &amp; Co. KG</t>
+          <t>Hörmann KG Verkaufsgesellschaft</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>https://www.krone-group.com</t>
+          <t>https://www.hoermann.de</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>+49 5977 935-0</t>
+          <t>+49 5204 915-0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Hörmann KG Verkaufsgesellschaft</t>
+          <t>Roto Frank Fenster- und Türtechnologie GmbH</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>https://www.hoermann.de</t>
+          <t>https://ftt.roto-frank.com</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>+49 5204 915-0</t>
+          <t>+49 711 7598-0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Roto Frank Fenster- und Türtechnologie GmbH</t>
+          <t>SIEGENIA-AUBI KG</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>https://ftt.roto-frank.com</t>
+          <t>https://www.siegenia.com</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>+49 711 7598-0</t>
+          <t>+49 271 3931-0</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SIEGENIA-AUBI KG</t>
+          <t>WAFIOS AG</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>https://www.siegenia.com</t>
+          <t>https://www.wafios.com</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>+49 271 3931-0</t>
+          <t>+49 7121 146-0</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>WAFIOS AG</t>
+          <t>Heller Maschinenfabrik GmbH (Gebr. Heller)</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>https://www.wafios.com</t>
+          <t>https://www.heller.biz</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>+49 7121 146-0</t>
+          <t>+49 7022 77-0</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Heller Maschinenfabrik GmbH (Gebr. Heller)</t>
+          <t>Alfred Kärcher SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>https://www.heller.biz</t>
+          <t>https://www.kaercher.com</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>+49 7022 77-0</t>
+          <t>+49 7195 14-0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Alfred Kärcher SE &amp; Co. KG</t>
+          <t>Ziehl-Abegg SE</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>https://www.kaercher.com</t>
+          <t>https://www.ziehl-abegg.com</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>+49 7195 14-0</t>
+          <t>+49 7940 16-0</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Ziehl-Abegg SE</t>
+          <t>fischerwerke GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>https://www.ziehl-abegg.com</t>
+          <t>https://www.fischer.de</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>+49 7940 16-0</t>
+          <t>+49 7443 12-0</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>fischerwerke GmbH &amp; Co. KG</t>
+          <t>Rittal GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>https://www.fischer.de</t>
+          <t>https://www.rittal.com</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>+49 7443 12-0</t>
+          <t>+49 2772 505-0</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Rittal GmbH &amp; Co. KG</t>
+          <t>Sto SE &amp; Co. KGaA</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>https://www.rittal.com</t>
+          <t>https://www.sto.de</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>+49 2772 505-0</t>
+          <t>+49 7744 57-0</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Sto SE &amp; Co. KGaA</t>
+          <t>WILO SE</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>https://www.sto.de</t>
+          <t>https://www.wilo.com</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>+49 7744 57-0</t>
+          <t>+49 231 4102-0</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>WILO SE</t>
+          <t>Festo SE &amp; Co. KG</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>https://www.wilo.com</t>
+          <t>https://www.festo.com</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>+49 231 4102-0</t>
+          <t>+49 711 347-0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Festo SE &amp; Co. KG</t>
+          <t>Vaillant GmbH</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>https://www.festo.com</t>
+          <t>https://www.vaillant.de</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>+49 711 347-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Vaillant GmbH</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>https://www.vaillant.de</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
           <t>+49 2191 18-0</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C38"/>
+  <autoFilter ref="A1:C37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1136,7 +1119,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>